<commit_message>
Mise à jour du suivi — 30/09/2026 23:40:12
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -689,17 +689,94 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>46295</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="5">
+        <v>2</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+      <c r="B24" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="5">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="3"/>
+      <c r="B25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
+      <c r="B28" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A13:A19"/>
+    <mergeCell ref="A22:A28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:40:16
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -714,8 +714,12 @@
       <c r="C23" s="5">
         <v>2</v>
       </c>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
+      <c r="D23" s="5">
+        <v>3</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:40:20
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -740,8 +740,12 @@
       <c r="C25" s="5">
         <v>1</v>
       </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
+      <c r="D25" s="5">
+        <v>1</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:40:25
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -755,8 +755,12 @@
       <c r="C26" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
+      <c r="D26" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:40:31
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -770,8 +770,12 @@
       <c r="C27" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
+      <c r="D27" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:41:00
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -714,12 +714,8 @@
       <c r="C23" s="5">
         <v>2</v>
       </c>
-      <c r="D23" s="5">
-        <v>3</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
@@ -740,12 +736,8 @@
       <c r="C25" s="5">
         <v>1</v>
       </c>
-      <c r="D25" s="5">
-        <v>1</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
@@ -755,12 +747,8 @@
       <c r="C26" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
@@ -770,12 +758,8 @@
       <c r="C27" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:41:05
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -714,8 +714,12 @@
       <c r="C23" s="5">
         <v>2</v>
       </c>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
+      <c r="D23" s="5">
+        <v>3</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 21:44:11
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -455,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -776,11 +776,95 @@
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
     </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <v>46296</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
+      <c r="B32" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="5">
+        <v>2</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="3"/>
+      <c r="B33" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="5">
+        <v>1</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="3"/>
+      <c r="B34" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="5">
+        <v>1</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="3"/>
+      <c r="B35" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="3"/>
+      <c r="B36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="3"/>
+      <c r="B37" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="A22:A28"/>
+    <mergeCell ref="A31:A37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 21:44:31
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>60min</t>
+  </si>
+  <si>
+    <t>Nouvelle action</t>
   </si>
 </sst>
 </file>
@@ -455,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -776,6 +779,8 @@
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
     </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>46296</v>
@@ -858,13 +863,22 @@
       </c>
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="3"/>
+      <c r="B38" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="A22:A28"/>
-    <mergeCell ref="A31:A37"/>
+    <mergeCell ref="A31:A38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 21:44:34
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>60min</t>
-  </si>
-  <si>
-    <t>Nouvelle action</t>
   </si>
 </sst>
 </file>
@@ -864,21 +861,13 @@
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="3"/>
-      <c r="B38" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="A22:A28"/>
-    <mergeCell ref="A31:A38"/>
+    <mergeCell ref="A31:A37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 21:44:50
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -803,8 +803,12 @@
       <c r="C32" s="5">
         <v>2</v>
       </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
+      <c r="D32" s="5">
+        <v>3</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:46:10
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="16">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -803,12 +803,8 @@
       <c r="C32" s="5">
         <v>2</v>
       </c>
-      <c r="D32" s="5">
-        <v>3</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 30/09/2026 23:52:15
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>60min</t>
+  </si>
+  <si>
+    <t>Nouvelle action</t>
   </si>
 </sst>
 </file>
@@ -582,50 +585,44 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
         <v>46294</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="5">
-        <v>2</v>
-      </c>
-      <c r="D14" s="5">
-        <v>4</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C15" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>7</v>
@@ -634,108 +631,112 @@
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C16" s="5">
         <v>1</v>
       </c>
       <c r="D16" s="5">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>15</v>
+        <v>10</v>
+      </c>
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="5">
+        <v>0.5</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="D18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="5" t="s">
+      <c r="C20" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
         <v>46295</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B23" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="5">
-        <v>2</v>
-      </c>
-      <c r="D23" s="5">
-        <v>3</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C24" s="5">
-        <v>1</v>
-      </c>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
+        <v>2</v>
+      </c>
+      <c r="D24" s="5">
+        <v>3</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C25" s="5">
         <v>1</v>
@@ -746,10 +747,10 @@
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="C26" s="5">
+        <v>1</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
@@ -757,7 +758,7 @@
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>12</v>
@@ -768,7 +769,7 @@
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>12</v>
@@ -776,43 +777,43 @@
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="3"/>
+      <c r="B29" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+    </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
         <v>46296</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B32" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-      <c r="B32" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" s="5">
-        <v>2</v>
-      </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C33" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" s="5"/>
       <c r="E33" s="5"/>
@@ -820,7 +821,7 @@
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C34" s="5">
         <v>1</v>
@@ -831,10 +832,10 @@
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="C35" s="5">
+        <v>1</v>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="5"/>
@@ -842,7 +843,7 @@
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>12</v>
@@ -853,7 +854,7 @@
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>12</v>
@@ -861,13 +862,23 @@
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="3"/>
+      <c r="B38" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+    </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A4:A10"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="A22:A28"/>
-    <mergeCell ref="A31:A37"/>
+    <mergeCell ref="A4:A11"/>
+    <mergeCell ref="A14:A20"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A32:A38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:06
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Nouvelle action</t>
+  </si>
+  <si>
+    <t>❌ Non fait</t>
   </si>
 </sst>
 </file>
@@ -815,8 +818,12 @@
       <c r="C33" s="5">
         <v>2</v>
       </c>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
+      <c r="D33" s="5">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:09
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>Nouvelle action</t>
-  </si>
-  <si>
-    <t>❌ Non fait</t>
   </si>
 </sst>
 </file>
@@ -818,12 +815,8 @@
       <c r="C33" s="5">
         <v>2</v>
       </c>
-      <c r="D33" s="5">
-        <v>0</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:13
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Nouvelle action</t>
+  </si>
+  <si>
+    <t>❌ Non fait</t>
   </si>
 </sst>
 </file>
@@ -815,8 +818,12 @@
       <c r="C33" s="5">
         <v>2</v>
       </c>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
+      <c r="D33" s="5">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:14
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -833,8 +833,12 @@
       <c r="C34" s="5">
         <v>1</v>
       </c>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
+      <c r="D34" s="5">
+        <v>0</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:16
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -848,8 +848,12 @@
       <c r="C35" s="5">
         <v>1</v>
       </c>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
+      <c r="D35" s="5">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:18
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>❌ Non fait</t>
+  </si>
+  <si>
+    <t>0min</t>
   </si>
 </sst>
 </file>
@@ -863,8 +866,12 @@
       <c r="C36" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
+      <c r="D36" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:20
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -881,8 +881,12 @@
       <c r="C37" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
+      <c r="D37" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:23
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -896,8 +896,12 @@
       <c r="C38" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
+      <c r="D38" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:25
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -896,12 +896,8 @@
       <c r="C38" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:32
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>0min</t>
+  </si>
+  <si>
+    <t>90min</t>
   </si>
 </sst>
 </file>
@@ -896,8 +899,12 @@
       <c r="C38" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
+      <c r="D38" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:37
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -906,12 +906,96 @@
         <v>7</v>
       </c>
     </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="3">
+        <v>46297</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="3"/>
+      <c r="B42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="5">
+        <v>2</v>
+      </c>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="3"/>
+      <c r="B43" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="5">
+        <v>1</v>
+      </c>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="3"/>
+      <c r="B44" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="5">
+        <v>1</v>
+      </c>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="3"/>
+      <c r="B45" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="3"/>
+      <c r="B46" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="3"/>
+      <c r="B47" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
     <mergeCell ref="A32:A38"/>
+    <mergeCell ref="A41:A47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:46:56
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>0min</t>
-  </si>
-  <si>
-    <t>90min</t>
   </si>
 </sst>
 </file>
@@ -467,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -884,12 +881,8 @@
       <c r="C37" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
@@ -899,103 +892,15 @@
       <c r="C38" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="3">
-        <v>46297</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-      <c r="B42" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" s="5">
-        <v>2</v>
-      </c>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-      <c r="B43" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C43" s="5">
-        <v>1</v>
-      </c>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="3"/>
-      <c r="B44" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" s="5">
-        <v>1</v>
-      </c>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="3"/>
-      <c r="B45" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="3"/>
-      <c r="B46" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-      <c r="B47" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
     <mergeCell ref="A32:A38"/>
-    <mergeCell ref="A41:A47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 01/10/2026 23:47:55
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>0min</t>
+  </si>
+  <si>
+    <t>90min</t>
   </si>
 </sst>
 </file>
@@ -464,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -881,8 +884,12 @@
       <c r="C37" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
+      <c r="D37" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
@@ -892,15 +899,105 @@
       <c r="C38" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
+      <c r="D38" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="3">
+        <v>46297</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="3"/>
+      <c r="B42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="5">
+        <v>2</v>
+      </c>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="3"/>
+      <c r="B43" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="5">
+        <v>1</v>
+      </c>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="3"/>
+      <c r="B44" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="5">
+        <v>1</v>
+      </c>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="3"/>
+      <c r="B45" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="3"/>
+      <c r="B46" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="3"/>
+      <c r="B47" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
     <mergeCell ref="A32:A38"/>
+    <mergeCell ref="A41:A47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 14/10/2026 11:59:10
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -991,13 +991,97 @@
       <c r="D47" s="5"/>
       <c r="E47" s="5"/>
     </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="3">
+        <v>46298</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="3"/>
+      <c r="B51" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" s="5">
+        <v>2</v>
+      </c>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="3"/>
+      <c r="B52" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" s="5">
+        <v>1</v>
+      </c>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="3"/>
+      <c r="B53" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" s="5">
+        <v>1</v>
+      </c>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="3"/>
+      <c r="B54" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="3"/>
+      <c r="B55" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="3"/>
+      <c r="B56" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
     <mergeCell ref="A32:A38"/>
     <mergeCell ref="A41:A47"/>
+    <mergeCell ref="A50:A56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 14/10/2026 11:59:45
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -991,6 +991,8 @@
       <c r="D47" s="5"/>
       <c r="E47" s="5"/>
     </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>46298</v>
@@ -1074,14 +1076,100 @@
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
     </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <v>46299</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="3"/>
+      <c r="B60" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" s="5">
+        <v>2</v>
+      </c>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="3"/>
+      <c r="B61" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C61" s="5">
+        <v>1</v>
+      </c>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="3"/>
+      <c r="B62" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" s="5">
+        <v>1</v>
+      </c>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="3"/>
+      <c r="B63" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="3"/>
+      <c r="B64" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="3"/>
+      <c r="B65" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
     <mergeCell ref="A32:A38"/>
     <mergeCell ref="A41:A47"/>
     <mergeCell ref="A50:A56"/>
+    <mergeCell ref="A59:A65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 14/10/2026 12:00:45
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -1161,8 +1161,858 @@
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
     </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="3">
+        <v>46300</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="3"/>
+      <c r="B69" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" s="5">
+        <v>2</v>
+      </c>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="3"/>
+      <c r="B70" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" s="5">
+        <v>1</v>
+      </c>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="3"/>
+      <c r="B71" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" s="5">
+        <v>1</v>
+      </c>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="3"/>
+      <c r="B72" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="3"/>
+      <c r="B73" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="3"/>
+      <c r="B74" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="3">
+        <v>46301</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="3"/>
+      <c r="B78" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C78" s="5">
+        <v>2</v>
+      </c>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="3"/>
+      <c r="B79" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C79" s="5">
+        <v>1</v>
+      </c>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="3"/>
+      <c r="B80" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C80" s="5">
+        <v>1</v>
+      </c>
+      <c r="D80" s="5"/>
+      <c r="E80" s="5"/>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="3"/>
+      <c r="B81" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="3"/>
+      <c r="B82" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="3"/>
+      <c r="B83" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="3">
+        <v>46302</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D86" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="3"/>
+      <c r="B87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" s="5">
+        <v>2</v>
+      </c>
+      <c r="D87" s="5"/>
+      <c r="E87" s="5"/>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="3"/>
+      <c r="B88" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C88" s="5">
+        <v>1</v>
+      </c>
+      <c r="D88" s="5"/>
+      <c r="E88" s="5"/>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="3"/>
+      <c r="B89" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C89" s="5">
+        <v>1</v>
+      </c>
+      <c r="D89" s="5"/>
+      <c r="E89" s="5"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="3"/>
+      <c r="B90" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="3"/>
+      <c r="B91" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C91" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D91" s="5"/>
+      <c r="E91" s="5"/>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="3"/>
+      <c r="B92" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="3">
+        <v>46303</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C95" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D95" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E95" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="3"/>
+      <c r="B96" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C96" s="5">
+        <v>2</v>
+      </c>
+      <c r="D96" s="5"/>
+      <c r="E96" s="5"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="3"/>
+      <c r="B97" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C97" s="5">
+        <v>1</v>
+      </c>
+      <c r="D97" s="5"/>
+      <c r="E97" s="5"/>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="3"/>
+      <c r="B98" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C98" s="5">
+        <v>1</v>
+      </c>
+      <c r="D98" s="5"/>
+      <c r="E98" s="5"/>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="3"/>
+      <c r="B99" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C99" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D99" s="5"/>
+      <c r="E99" s="5"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="3"/>
+      <c r="B100" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C100" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D100" s="5"/>
+      <c r="E100" s="5"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="3"/>
+      <c r="B101" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D101" s="5"/>
+      <c r="E101" s="5"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="3">
+        <v>46304</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E104" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="3"/>
+      <c r="B105" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C105" s="5">
+        <v>2</v>
+      </c>
+      <c r="D105" s="5"/>
+      <c r="E105" s="5"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="3"/>
+      <c r="B106" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C106" s="5">
+        <v>1</v>
+      </c>
+      <c r="D106" s="5"/>
+      <c r="E106" s="5"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="3"/>
+      <c r="B107" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C107" s="5">
+        <v>1</v>
+      </c>
+      <c r="D107" s="5"/>
+      <c r="E107" s="5"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="3"/>
+      <c r="B108" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C108" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D108" s="5"/>
+      <c r="E108" s="5"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="3"/>
+      <c r="B109" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C109" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D109" s="5"/>
+      <c r="E109" s="5"/>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="3"/>
+      <c r="B110" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D110" s="5"/>
+      <c r="E110" s="5"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="3">
+        <v>46305</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C113" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E113" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="3"/>
+      <c r="B114" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C114" s="5">
+        <v>2</v>
+      </c>
+      <c r="D114" s="5"/>
+      <c r="E114" s="5"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="3"/>
+      <c r="B115" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C115" s="5">
+        <v>1</v>
+      </c>
+      <c r="D115" s="5"/>
+      <c r="E115" s="5"/>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="3"/>
+      <c r="B116" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C116" s="5">
+        <v>1</v>
+      </c>
+      <c r="D116" s="5"/>
+      <c r="E116" s="5"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" s="3"/>
+      <c r="B117" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C117" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5"/>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="3"/>
+      <c r="B118" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C118" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D118" s="5"/>
+      <c r="E118" s="5"/>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" s="3"/>
+      <c r="B119" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C119" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D119" s="5"/>
+      <c r="E119" s="5"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" s="3">
+        <v>46306</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" s="3"/>
+      <c r="B123" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C123" s="5">
+        <v>2</v>
+      </c>
+      <c r="D123" s="5"/>
+      <c r="E123" s="5"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" s="3"/>
+      <c r="B124" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C124" s="5">
+        <v>1</v>
+      </c>
+      <c r="D124" s="5"/>
+      <c r="E124" s="5"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" s="3"/>
+      <c r="B125" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C125" s="5">
+        <v>1</v>
+      </c>
+      <c r="D125" s="5"/>
+      <c r="E125" s="5"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" s="3"/>
+      <c r="B126" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D126" s="5"/>
+      <c r="E126" s="5"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" s="3"/>
+      <c r="B127" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C127" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D127" s="5"/>
+      <c r="E127" s="5"/>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" s="3"/>
+      <c r="B128" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D128" s="5"/>
+      <c r="E128" s="5"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" s="3">
+        <v>46307</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" s="3"/>
+      <c r="B132" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C132" s="5">
+        <v>2</v>
+      </c>
+      <c r="D132" s="5"/>
+      <c r="E132" s="5"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" s="3"/>
+      <c r="B133" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C133" s="5">
+        <v>1</v>
+      </c>
+      <c r="D133" s="5"/>
+      <c r="E133" s="5"/>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" s="3"/>
+      <c r="B134" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C134" s="5">
+        <v>1</v>
+      </c>
+      <c r="D134" s="5"/>
+      <c r="E134" s="5"/>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" s="3"/>
+      <c r="B135" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D135" s="5"/>
+      <c r="E135" s="5"/>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" s="3"/>
+      <c r="B136" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D136" s="5"/>
+      <c r="E136" s="5"/>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" s="3"/>
+      <c r="B137" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D137" s="5"/>
+      <c r="E137" s="5"/>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" s="3">
+        <v>46308</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E140" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" s="3"/>
+      <c r="B141" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C141" s="5">
+        <v>2</v>
+      </c>
+      <c r="D141" s="5"/>
+      <c r="E141" s="5"/>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" s="3"/>
+      <c r="B142" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C142" s="5">
+        <v>1</v>
+      </c>
+      <c r="D142" s="5"/>
+      <c r="E142" s="5"/>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" s="3"/>
+      <c r="B143" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C143" s="5">
+        <v>1</v>
+      </c>
+      <c r="D143" s="5"/>
+      <c r="E143" s="5"/>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" s="3"/>
+      <c r="B144" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C144" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D144" s="5"/>
+      <c r="E144" s="5"/>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" s="3"/>
+      <c r="B145" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C145" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D145" s="5"/>
+      <c r="E145" s="5"/>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A146" s="3"/>
+      <c r="B146" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C146" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D146" s="5"/>
+      <c r="E146" s="5"/>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" s="3">
+        <v>46309</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C149" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D149" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E149" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" s="3"/>
+      <c r="B150" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C150" s="5">
+        <v>2</v>
+      </c>
+      <c r="D150" s="5"/>
+      <c r="E150" s="5"/>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" s="3"/>
+      <c r="B151" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C151" s="5">
+        <v>1</v>
+      </c>
+      <c r="D151" s="5"/>
+      <c r="E151" s="5"/>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" s="3"/>
+      <c r="B152" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C152" s="5">
+        <v>1</v>
+      </c>
+      <c r="D152" s="5"/>
+      <c r="E152" s="5"/>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" s="3"/>
+      <c r="B153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C153" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D153" s="5"/>
+      <c r="E153" s="5"/>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" s="3"/>
+      <c r="B154" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C154" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D154" s="5"/>
+      <c r="E154" s="5"/>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" s="3"/>
+      <c r="B155" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C155" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D155" s="5"/>
+      <c r="E155" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="17">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -1170,6 +2020,16 @@
     <mergeCell ref="A41:A47"/>
     <mergeCell ref="A50:A56"/>
     <mergeCell ref="A59:A65"/>
+    <mergeCell ref="A68:A74"/>
+    <mergeCell ref="A77:A83"/>
+    <mergeCell ref="A86:A92"/>
+    <mergeCell ref="A95:A101"/>
+    <mergeCell ref="A104:A110"/>
+    <mergeCell ref="A113:A119"/>
+    <mergeCell ref="A122:A128"/>
+    <mergeCell ref="A131:A137"/>
+    <mergeCell ref="A140:A146"/>
+    <mergeCell ref="A149:A155"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 16/10/2026 17:04:51
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2011,8 +2011,91 @@
       <c r="D155" s="5"/>
       <c r="E155" s="5"/>
     </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" s="3">
+        <v>46310</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C158" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" s="3"/>
+      <c r="B159" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C159" s="5">
+        <v>2</v>
+      </c>
+      <c r="D159" s="5"/>
+      <c r="E159" s="5"/>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" s="3"/>
+      <c r="B160" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C160" s="5">
+        <v>1</v>
+      </c>
+      <c r="D160" s="5"/>
+      <c r="E160" s="5"/>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" s="3"/>
+      <c r="B161" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C161" s="5">
+        <v>1</v>
+      </c>
+      <c r="D161" s="5"/>
+      <c r="E161" s="5"/>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" s="3"/>
+      <c r="B162" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C162" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D162" s="5"/>
+      <c r="E162" s="5"/>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" s="3"/>
+      <c r="B163" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C163" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D163" s="5"/>
+      <c r="E163" s="5"/>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" s="3"/>
+      <c r="B164" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C164" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D164" s="5"/>
+      <c r="E164" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2030,6 +2113,7 @@
     <mergeCell ref="A131:A137"/>
     <mergeCell ref="A140:A146"/>
     <mergeCell ref="A149:A155"/>
+    <mergeCell ref="A158:A164"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 16/10/2026 17:05:03
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2011,6 +2011,8 @@
       <c r="D155" s="5"/>
       <c r="E155" s="5"/>
     </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="3">
         <v>46310</v>
@@ -2091,8 +2093,12 @@
       <c r="C164" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D164" s="5"/>
-      <c r="E164" s="5"/>
+      <c r="D164" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E164" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="18">

</xml_diff>

<commit_message>
Mise à jour du suivi — 16/10/2026 17:05:23
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E173"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2100,8 +2100,91 @@
         <v>7</v>
       </c>
     </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" s="3">
+        <v>46311</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C167" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D167" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E167" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" s="3"/>
+      <c r="B168" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C168" s="5">
+        <v>2</v>
+      </c>
+      <c r="D168" s="5"/>
+      <c r="E168" s="5"/>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" s="3"/>
+      <c r="B169" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C169" s="5">
+        <v>1</v>
+      </c>
+      <c r="D169" s="5"/>
+      <c r="E169" s="5"/>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" s="3"/>
+      <c r="B170" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C170" s="5">
+        <v>1</v>
+      </c>
+      <c r="D170" s="5"/>
+      <c r="E170" s="5"/>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" s="3"/>
+      <c r="B171" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C171" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D171" s="5"/>
+      <c r="E171" s="5"/>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" s="3"/>
+      <c r="B172" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C172" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D172" s="5"/>
+      <c r="E172" s="5"/>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" s="3"/>
+      <c r="B173" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C173" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D173" s="5"/>
+      <c r="E173" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2120,6 +2203,7 @@
     <mergeCell ref="A140:A146"/>
     <mergeCell ref="A149:A155"/>
     <mergeCell ref="A158:A164"/>
+    <mergeCell ref="A167:A173"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 16/10/2026 17:36:03
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2100,6 +2100,8 @@
         <v>7</v>
       </c>
     </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="3">
         <v>46311</v>
@@ -2125,8 +2127,12 @@
       <c r="C168" s="5">
         <v>2</v>
       </c>
-      <c r="D168" s="5"/>
-      <c r="E168" s="5"/>
+      <c r="D168" s="5">
+        <v>2</v>
+      </c>
+      <c r="E168" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 17/10/2026 18:02:29
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E173"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2189,8 +2189,91 @@
       <c r="D173" s="5"/>
       <c r="E173" s="5"/>
     </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" s="3">
+        <v>46312</v>
+      </c>
+      <c r="B176" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C176" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D176" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E176" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" s="3"/>
+      <c r="B177" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C177" s="5">
+        <v>2</v>
+      </c>
+      <c r="D177" s="5"/>
+      <c r="E177" s="5"/>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" s="3"/>
+      <c r="B178" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C178" s="5">
+        <v>1</v>
+      </c>
+      <c r="D178" s="5"/>
+      <c r="E178" s="5"/>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" s="3"/>
+      <c r="B179" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C179" s="5">
+        <v>1</v>
+      </c>
+      <c r="D179" s="5"/>
+      <c r="E179" s="5"/>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" s="3"/>
+      <c r="B180" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C180" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D180" s="5"/>
+      <c r="E180" s="5"/>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" s="3"/>
+      <c r="B181" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C181" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D181" s="5"/>
+      <c r="E181" s="5"/>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" s="3"/>
+      <c r="B182" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C182" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D182" s="5"/>
+      <c r="E182" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2210,6 +2293,7 @@
     <mergeCell ref="A149:A155"/>
     <mergeCell ref="A158:A164"/>
     <mergeCell ref="A167:A173"/>
+    <mergeCell ref="A176:A182"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 17/10/2026 18:02:33
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2189,6 +2189,8 @@
       <c r="D173" s="5"/>
       <c r="E173" s="5"/>
     </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="3">
         <v>46312</v>
@@ -2214,8 +2216,12 @@
       <c r="C177" s="5">
         <v>2</v>
       </c>
-      <c r="D177" s="5"/>
-      <c r="E177" s="5"/>
+      <c r="D177" s="5">
+        <v>1</v>
+      </c>
+      <c r="E177" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 17/10/2026 18:02:38
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2216,12 +2216,8 @@
       <c r="C177" s="5">
         <v>2</v>
       </c>
-      <c r="D177" s="5">
-        <v>1</v>
-      </c>
-      <c r="E177" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="D177" s="5"/>
+      <c r="E177" s="5"/>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 17/10/2026 18:02:46
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2249,8 +2249,12 @@
       <c r="C180" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D180" s="5"/>
-      <c r="E180" s="5"/>
+      <c r="D180" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E180" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 18/10/2026 15:25:31
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E182"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2278,8 +2278,91 @@
       <c r="D182" s="5"/>
       <c r="E182" s="5"/>
     </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" s="3">
+        <v>46313</v>
+      </c>
+      <c r="B185" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C185" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D185" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E185" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" s="3"/>
+      <c r="B186" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C186" s="5">
+        <v>2</v>
+      </c>
+      <c r="D186" s="5"/>
+      <c r="E186" s="5"/>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" s="3"/>
+      <c r="B187" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C187" s="5">
+        <v>1</v>
+      </c>
+      <c r="D187" s="5"/>
+      <c r="E187" s="5"/>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" s="3"/>
+      <c r="B188" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C188" s="5">
+        <v>1</v>
+      </c>
+      <c r="D188" s="5"/>
+      <c r="E188" s="5"/>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" s="3"/>
+      <c r="B189" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C189" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D189" s="5"/>
+      <c r="E189" s="5"/>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" s="3"/>
+      <c r="B190" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C190" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D190" s="5"/>
+      <c r="E190" s="5"/>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A191" s="3"/>
+      <c r="B191" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C191" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D191" s="5"/>
+      <c r="E191" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2300,6 +2383,7 @@
     <mergeCell ref="A158:A164"/>
     <mergeCell ref="A167:A173"/>
     <mergeCell ref="A176:A182"/>
+    <mergeCell ref="A185:A191"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:07:34
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2278,6 +2278,8 @@
       <c r="D182" s="5"/>
       <c r="E182" s="5"/>
     </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="3">
         <v>46313</v>
@@ -2361,8 +2363,91 @@
       <c r="D191" s="5"/>
       <c r="E191" s="5"/>
     </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" s="3">
+        <v>46314</v>
+      </c>
+      <c r="B194" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C194" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E194" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" s="3"/>
+      <c r="B195" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C195" s="5">
+        <v>2</v>
+      </c>
+      <c r="D195" s="5"/>
+      <c r="E195" s="5"/>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" s="3"/>
+      <c r="B196" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C196" s="5">
+        <v>1</v>
+      </c>
+      <c r="D196" s="5"/>
+      <c r="E196" s="5"/>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" s="3"/>
+      <c r="B197" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C197" s="5">
+        <v>1</v>
+      </c>
+      <c r="D197" s="5"/>
+      <c r="E197" s="5"/>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A198" s="3"/>
+      <c r="B198" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C198" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D198" s="5"/>
+      <c r="E198" s="5"/>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" s="3"/>
+      <c r="B199" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C199" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D199" s="5"/>
+      <c r="E199" s="5"/>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" s="3"/>
+      <c r="B200" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C200" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D200" s="5"/>
+      <c r="E200" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2384,6 +2469,7 @@
     <mergeCell ref="A167:A173"/>
     <mergeCell ref="A176:A182"/>
     <mergeCell ref="A185:A191"/>
+    <mergeCell ref="A194:A200"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:07:38
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:E209"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2363,6 +2363,8 @@
       <c r="D191" s="5"/>
       <c r="E191" s="5"/>
     </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="3">
         <v>46314</v>
@@ -2446,8 +2448,91 @@
       <c r="D200" s="5"/>
       <c r="E200" s="5"/>
     </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" s="3">
+        <v>46315</v>
+      </c>
+      <c r="B203" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C203" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D203" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E203" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" s="3"/>
+      <c r="B204" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C204" s="5">
+        <v>2</v>
+      </c>
+      <c r="D204" s="5"/>
+      <c r="E204" s="5"/>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" s="3"/>
+      <c r="B205" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C205" s="5">
+        <v>1</v>
+      </c>
+      <c r="D205" s="5"/>
+      <c r="E205" s="5"/>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" s="3"/>
+      <c r="B206" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C206" s="5">
+        <v>1</v>
+      </c>
+      <c r="D206" s="5"/>
+      <c r="E206" s="5"/>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" s="3"/>
+      <c r="B207" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C207" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D207" s="5"/>
+      <c r="E207" s="5"/>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" s="3"/>
+      <c r="B208" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C208" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D208" s="5"/>
+      <c r="E208" s="5"/>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" s="3"/>
+      <c r="B209" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C209" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D209" s="5"/>
+      <c r="E209" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2470,6 +2555,7 @@
     <mergeCell ref="A176:A182"/>
     <mergeCell ref="A185:A191"/>
     <mergeCell ref="A194:A200"/>
+    <mergeCell ref="A203:A209"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:07:41
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E209"/>
+  <dimension ref="A1:E218"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2448,6 +2448,8 @@
       <c r="D200" s="5"/>
       <c r="E200" s="5"/>
     </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="3">
         <v>46315</v>
@@ -2531,8 +2533,91 @@
       <c r="D209" s="5"/>
       <c r="E209" s="5"/>
     </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" s="3">
+        <v>46316</v>
+      </c>
+      <c r="B212" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C212" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D212" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E212" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" s="3"/>
+      <c r="B213" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C213" s="5">
+        <v>2</v>
+      </c>
+      <c r="D213" s="5"/>
+      <c r="E213" s="5"/>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" s="3"/>
+      <c r="B214" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C214" s="5">
+        <v>1</v>
+      </c>
+      <c r="D214" s="5"/>
+      <c r="E214" s="5"/>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" s="3"/>
+      <c r="B215" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C215" s="5">
+        <v>1</v>
+      </c>
+      <c r="D215" s="5"/>
+      <c r="E215" s="5"/>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" s="3"/>
+      <c r="B216" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C216" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D216" s="5"/>
+      <c r="E216" s="5"/>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" s="3"/>
+      <c r="B217" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C217" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D217" s="5"/>
+      <c r="E217" s="5"/>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" s="3"/>
+      <c r="B218" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C218" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D218" s="5"/>
+      <c r="E218" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2556,6 +2641,7 @@
     <mergeCell ref="A185:A191"/>
     <mergeCell ref="A194:A200"/>
     <mergeCell ref="A203:A209"/>
+    <mergeCell ref="A212:A218"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:07:43
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E218"/>
+  <dimension ref="A1:E227"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2533,6 +2533,8 @@
       <c r="D209" s="5"/>
       <c r="E209" s="5"/>
     </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="3">
         <v>46316</v>
@@ -2616,8 +2618,91 @@
       <c r="D218" s="5"/>
       <c r="E218" s="5"/>
     </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A221" s="3">
+        <v>46317</v>
+      </c>
+      <c r="B221" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C221" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D221" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E221" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A222" s="3"/>
+      <c r="B222" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C222" s="5">
+        <v>2</v>
+      </c>
+      <c r="D222" s="5"/>
+      <c r="E222" s="5"/>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A223" s="3"/>
+      <c r="B223" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C223" s="5">
+        <v>1</v>
+      </c>
+      <c r="D223" s="5"/>
+      <c r="E223" s="5"/>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A224" s="3"/>
+      <c r="B224" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C224" s="5">
+        <v>1</v>
+      </c>
+      <c r="D224" s="5"/>
+      <c r="E224" s="5"/>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A225" s="3"/>
+      <c r="B225" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C225" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D225" s="5"/>
+      <c r="E225" s="5"/>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A226" s="3"/>
+      <c r="B226" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C226" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D226" s="5"/>
+      <c r="E226" s="5"/>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A227" s="3"/>
+      <c r="B227" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C227" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D227" s="5"/>
+      <c r="E227" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="25">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2642,6 +2727,7 @@
     <mergeCell ref="A194:A200"/>
     <mergeCell ref="A203:A209"/>
     <mergeCell ref="A212:A218"/>
+    <mergeCell ref="A221:A227"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:07:46
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E227"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2618,6 +2618,8 @@
       <c r="D218" s="5"/>
       <c r="E218" s="5"/>
     </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="3">
         <v>46317</v>
@@ -2701,8 +2703,91 @@
       <c r="D227" s="5"/>
       <c r="E227" s="5"/>
     </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A230" s="3">
+        <v>46318</v>
+      </c>
+      <c r="B230" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C230" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D230" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E230" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A231" s="3"/>
+      <c r="B231" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C231" s="5">
+        <v>2</v>
+      </c>
+      <c r="D231" s="5"/>
+      <c r="E231" s="5"/>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A232" s="3"/>
+      <c r="B232" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C232" s="5">
+        <v>1</v>
+      </c>
+      <c r="D232" s="5"/>
+      <c r="E232" s="5"/>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A233" s="3"/>
+      <c r="B233" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C233" s="5">
+        <v>1</v>
+      </c>
+      <c r="D233" s="5"/>
+      <c r="E233" s="5"/>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A234" s="3"/>
+      <c r="B234" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C234" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D234" s="5"/>
+      <c r="E234" s="5"/>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A235" s="3"/>
+      <c r="B235" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C235" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D235" s="5"/>
+      <c r="E235" s="5"/>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A236" s="3"/>
+      <c r="B236" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C236" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D236" s="5"/>
+      <c r="E236" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="26">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2728,6 +2813,7 @@
     <mergeCell ref="A203:A209"/>
     <mergeCell ref="A212:A218"/>
     <mergeCell ref="A221:A227"/>
+    <mergeCell ref="A230:A236"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:07:49
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E245"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2703,6 +2703,8 @@
       <c r="D227" s="5"/>
       <c r="E227" s="5"/>
     </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="3">
         <v>46318</v>
@@ -2786,8 +2788,91 @@
       <c r="D236" s="5"/>
       <c r="E236" s="5"/>
     </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A239" s="3">
+        <v>46319</v>
+      </c>
+      <c r="B239" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C239" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D239" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E239" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A240" s="3"/>
+      <c r="B240" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C240" s="5">
+        <v>2</v>
+      </c>
+      <c r="D240" s="5"/>
+      <c r="E240" s="5"/>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A241" s="3"/>
+      <c r="B241" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C241" s="5">
+        <v>1</v>
+      </c>
+      <c r="D241" s="5"/>
+      <c r="E241" s="5"/>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A242" s="3"/>
+      <c r="B242" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C242" s="5">
+        <v>1</v>
+      </c>
+      <c r="D242" s="5"/>
+      <c r="E242" s="5"/>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A243" s="3"/>
+      <c r="B243" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C243" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D243" s="5"/>
+      <c r="E243" s="5"/>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A244" s="3"/>
+      <c r="B244" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C244" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D244" s="5"/>
+      <c r="E244" s="5"/>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A245" s="3"/>
+      <c r="B245" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C245" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D245" s="5"/>
+      <c r="E245" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2814,6 +2899,7 @@
     <mergeCell ref="A212:A218"/>
     <mergeCell ref="A221:A227"/>
     <mergeCell ref="A230:A236"/>
+    <mergeCell ref="A239:A245"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:07:54
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -467,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E245"/>
+  <dimension ref="A1:E254"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2788,6 +2788,8 @@
       <c r="D236" s="5"/>
       <c r="E236" s="5"/>
     </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="3">
         <v>46319</v>
@@ -2871,8 +2873,91 @@
       <c r="D245" s="5"/>
       <c r="E245" s="5"/>
     </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A248" s="3">
+        <v>46320</v>
+      </c>
+      <c r="B248" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C248" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D248" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E248" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A249" s="3"/>
+      <c r="B249" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C249" s="5">
+        <v>2</v>
+      </c>
+      <c r="D249" s="5"/>
+      <c r="E249" s="5"/>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A250" s="3"/>
+      <c r="B250" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C250" s="5">
+        <v>1</v>
+      </c>
+      <c r="D250" s="5"/>
+      <c r="E250" s="5"/>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A251" s="3"/>
+      <c r="B251" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C251" s="5">
+        <v>1</v>
+      </c>
+      <c r="D251" s="5"/>
+      <c r="E251" s="5"/>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A252" s="3"/>
+      <c r="B252" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C252" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D252" s="5"/>
+      <c r="E252" s="5"/>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A253" s="3"/>
+      <c r="B253" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C253" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D253" s="5"/>
+      <c r="E253" s="5"/>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A254" s="3"/>
+      <c r="B254" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C254" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D254" s="5"/>
+      <c r="E254" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2900,6 +2985,7 @@
     <mergeCell ref="A221:A227"/>
     <mergeCell ref="A230:A236"/>
     <mergeCell ref="A239:A245"/>
+    <mergeCell ref="A248:A254"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 14:08:09
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2873,6 +2873,8 @@
       <c r="D245" s="5"/>
       <c r="E245" s="5"/>
     </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="3">
         <v>46320</v>
@@ -2920,8 +2922,12 @@
       <c r="C251" s="5">
         <v>1</v>
       </c>
-      <c r="D251" s="5"/>
-      <c r="E251" s="5"/>
+      <c r="D251" s="5">
+        <v>1</v>
+      </c>
+      <c r="E251" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:14:02
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -557,11 +557,11 @@
       <c r="C8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>12</v>
+      <c r="D8" s="5">
+        <v>1</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:14:04
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -572,11 +572,11 @@
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>12</v>
+      <c r="D9" s="5">
+        <v>1</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:14:06
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -74,10 +74,10 @@
     <t>🚀 Projet personnel</t>
   </si>
   <si>
-    <t>60min</t>
+    <t>Nouvelle action</t>
   </si>
   <si>
-    <t>Nouvelle action</t>
+    <t>60min</t>
   </si>
   <si>
     <t>❌ Non fait</t>
@@ -587,17 +587,17 @@
       <c r="C10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>15</v>
+      <c r="D10" s="5">
+        <v>2</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
@@ -676,7 +676,7 @@
         <v>12</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>7</v>
@@ -702,7 +702,7 @@
         <v>12</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:14:32
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -675,11 +675,11 @@
       <c r="C18" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>16</v>
+      <c r="D18" s="5">
+        <v>2</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:14:35
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>Nouvelle action</t>
-  </si>
-  <si>
-    <t>60min</t>
   </si>
   <si>
     <t>❌ Non fait</t>
@@ -701,11 +698,11 @@
       <c r="C20" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>16</v>
+      <c r="D20" s="5">
+        <v>1</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25"/>
@@ -828,7 +825,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -843,7 +840,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -858,7 +855,7 @@
         <v>0</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -870,10 +867,10 @@
         <v>12</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -885,10 +882,10 @@
         <v>12</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -900,7 +897,7 @@
         <v>12</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:14:53
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -83,7 +83,7 @@
     <t>0min</t>
   </si>
   <si>
-    <t>90min</t>
+    <t>3min</t>
   </si>
 </sst>
 </file>
@@ -900,7 +900,7 @@
         <v>18</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:14:55
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>0min</t>
-  </si>
-  <si>
-    <t>3min</t>
   </si>
 </sst>
 </file>
@@ -896,8 +893,8 @@
       <c r="C38" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="5" t="s">
-        <v>18</v>
+      <c r="D38" s="5">
+        <v>3</v>
       </c>
       <c r="E38" s="5" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:15:30
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2087,11 +2087,11 @@
       <c r="C164" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D164" s="5" t="s">
-        <v>12</v>
+      <c r="D164" s="5">
+        <v>1</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:15:43
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2243,11 +2243,11 @@
       <c r="C180" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D180" s="5" t="s">
-        <v>12</v>
+      <c r="D180" s="5">
+        <v>1</v>
       </c>
       <c r="E180" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:16:53
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>0min</t>
+  </si>
+  <si>
+    <t>&amp;</t>
   </si>
 </sst>
 </file>
@@ -2931,7 +2934,9 @@
       <c r="C252" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D252" s="5"/>
+      <c r="D252" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="E252" s="5"/>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:16:56
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>0min</t>
-  </si>
-  <si>
-    <t>&amp;</t>
   </si>
 </sst>
 </file>
@@ -2934,10 +2931,12 @@
       <c r="C252" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D252" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E252" s="5"/>
+      <c r="D252" s="5">
+        <v>1</v>
+      </c>
+      <c r="E252" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:17:05
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2928,14 +2928,14 @@
       <c r="B252" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C252" s="5" t="s">
-        <v>12</v>
+      <c r="C252" s="5">
+        <v>1</v>
       </c>
       <c r="D252" s="5">
         <v>1</v>
       </c>
       <c r="E252" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:17:08
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>0min</t>
+  </si>
+  <si>
+    <t>&amp;</t>
   </si>
 </sst>
 </file>
@@ -2944,7 +2947,7 @@
         <v>13</v>
       </c>
       <c r="C253" s="5" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D253" s="5"/>
       <c r="E253" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:17:10
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>0min</t>
-  </si>
-  <si>
-    <t>&amp;</t>
   </si>
 </sst>
 </file>
@@ -2946,8 +2943,8 @@
       <c r="B253" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C253" s="5" t="s">
-        <v>18</v>
+      <c r="C253" s="5">
+        <v>1</v>
       </c>
       <c r="D253" s="5"/>
       <c r="E253" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:18:03
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2329,8 +2329,8 @@
       <c r="B189" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C189" s="5" t="s">
-        <v>12</v>
+      <c r="C189" s="5">
+        <v>1</v>
       </c>
       <c r="D189" s="5"/>
       <c r="E189" s="5"/>
@@ -2340,8 +2340,8 @@
       <c r="B190" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C190" s="5" t="s">
-        <v>12</v>
+      <c r="C190" s="5">
+        <v>1</v>
       </c>
       <c r="D190" s="5"/>
       <c r="E190" s="5"/>
@@ -2351,8 +2351,8 @@
       <c r="B191" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C191" s="5" t="s">
-        <v>12</v>
+      <c r="C191" s="5">
+        <v>1</v>
       </c>
       <c r="D191" s="5"/>
       <c r="E191" s="5"/>
@@ -2414,8 +2414,8 @@
       <c r="B198" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C198" s="5" t="s">
-        <v>12</v>
+      <c r="C198" s="5">
+        <v>1</v>
       </c>
       <c r="D198" s="5"/>
       <c r="E198" s="5"/>
@@ -2425,8 +2425,8 @@
       <c r="B199" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C199" s="5" t="s">
-        <v>12</v>
+      <c r="C199" s="5">
+        <v>1</v>
       </c>
       <c r="D199" s="5"/>
       <c r="E199" s="5"/>
@@ -2436,8 +2436,8 @@
       <c r="B200" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C200" s="5" t="s">
-        <v>12</v>
+      <c r="C200" s="5">
+        <v>1</v>
       </c>
       <c r="D200" s="5"/>
       <c r="E200" s="5"/>
@@ -2499,8 +2499,8 @@
       <c r="B207" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C207" s="5" t="s">
-        <v>12</v>
+      <c r="C207" s="5">
+        <v>1</v>
       </c>
       <c r="D207" s="5"/>
       <c r="E207" s="5"/>
@@ -2510,8 +2510,8 @@
       <c r="B208" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C208" s="5" t="s">
-        <v>12</v>
+      <c r="C208" s="5">
+        <v>1</v>
       </c>
       <c r="D208" s="5"/>
       <c r="E208" s="5"/>
@@ -2521,8 +2521,8 @@
       <c r="B209" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C209" s="5" t="s">
-        <v>12</v>
+      <c r="C209" s="5">
+        <v>1</v>
       </c>
       <c r="D209" s="5"/>
       <c r="E209" s="5"/>
@@ -2584,8 +2584,8 @@
       <c r="B216" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C216" s="5" t="s">
-        <v>12</v>
+      <c r="C216" s="5">
+        <v>1</v>
       </c>
       <c r="D216" s="5"/>
       <c r="E216" s="5"/>
@@ -2595,8 +2595,8 @@
       <c r="B217" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C217" s="5" t="s">
-        <v>12</v>
+      <c r="C217" s="5">
+        <v>1</v>
       </c>
       <c r="D217" s="5"/>
       <c r="E217" s="5"/>
@@ -2606,8 +2606,8 @@
       <c r="B218" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C218" s="5" t="s">
-        <v>12</v>
+      <c r="C218" s="5">
+        <v>1</v>
       </c>
       <c r="D218" s="5"/>
       <c r="E218" s="5"/>
@@ -2669,8 +2669,8 @@
       <c r="B225" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C225" s="5" t="s">
-        <v>12</v>
+      <c r="C225" s="5">
+        <v>1</v>
       </c>
       <c r="D225" s="5"/>
       <c r="E225" s="5"/>
@@ -2680,8 +2680,8 @@
       <c r="B226" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C226" s="5" t="s">
-        <v>12</v>
+      <c r="C226" s="5">
+        <v>1</v>
       </c>
       <c r="D226" s="5"/>
       <c r="E226" s="5"/>
@@ -2691,8 +2691,8 @@
       <c r="B227" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C227" s="5" t="s">
-        <v>12</v>
+      <c r="C227" s="5">
+        <v>1</v>
       </c>
       <c r="D227" s="5"/>
       <c r="E227" s="5"/>
@@ -2754,8 +2754,8 @@
       <c r="B234" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C234" s="5" t="s">
-        <v>12</v>
+      <c r="C234" s="5">
+        <v>1</v>
       </c>
       <c r="D234" s="5"/>
       <c r="E234" s="5"/>
@@ -2765,8 +2765,8 @@
       <c r="B235" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C235" s="5" t="s">
-        <v>12</v>
+      <c r="C235" s="5">
+        <v>1</v>
       </c>
       <c r="D235" s="5"/>
       <c r="E235" s="5"/>
@@ -2776,8 +2776,8 @@
       <c r="B236" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C236" s="5" t="s">
-        <v>12</v>
+      <c r="C236" s="5">
+        <v>1</v>
       </c>
       <c r="D236" s="5"/>
       <c r="E236" s="5"/>
@@ -2839,8 +2839,8 @@
       <c r="B243" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C243" s="5" t="s">
-        <v>12</v>
+      <c r="C243" s="5">
+        <v>1</v>
       </c>
       <c r="D243" s="5"/>
       <c r="E243" s="5"/>
@@ -2850,8 +2850,8 @@
       <c r="B244" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C244" s="5" t="s">
-        <v>12</v>
+      <c r="C244" s="5">
+        <v>1</v>
       </c>
       <c r="D244" s="5"/>
       <c r="E244" s="5"/>
@@ -2861,8 +2861,8 @@
       <c r="B245" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C245" s="5" t="s">
-        <v>12</v>
+      <c r="C245" s="5">
+        <v>1</v>
       </c>
       <c r="D245" s="5"/>
       <c r="E245" s="5"/>
@@ -2954,8 +2954,8 @@
       <c r="B254" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C254" s="5" t="s">
-        <v>12</v>
+      <c r="C254" s="5">
+        <v>1</v>
       </c>
       <c r="D254" s="5"/>
       <c r="E254" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:18:25
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2240,14 +2240,14 @@
       <c r="B180" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C180" s="5" t="s">
-        <v>12</v>
+      <c r="C180" s="5">
+        <v>1</v>
       </c>
       <c r="D180" s="5">
         <v>1</v>
       </c>
       <c r="E180" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
@@ -2255,8 +2255,8 @@
       <c r="B181" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C181" s="5" t="s">
-        <v>12</v>
+      <c r="C181" s="5">
+        <v>1</v>
       </c>
       <c r="D181" s="5"/>
       <c r="E181" s="5"/>
@@ -2266,8 +2266,8 @@
       <c r="B182" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C182" s="5" t="s">
-        <v>12</v>
+      <c r="C182" s="5">
+        <v>1</v>
       </c>
       <c r="D182" s="5"/>
       <c r="E182" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:18:33
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2155,8 +2155,8 @@
       <c r="B171" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C171" s="5" t="s">
-        <v>12</v>
+      <c r="C171" s="5">
+        <v>1</v>
       </c>
       <c r="D171" s="5"/>
       <c r="E171" s="5"/>
@@ -2166,8 +2166,8 @@
       <c r="B172" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C172" s="5" t="s">
-        <v>12</v>
+      <c r="C172" s="5">
+        <v>1</v>
       </c>
       <c r="D172" s="5"/>
       <c r="E172" s="5"/>
@@ -2177,8 +2177,8 @@
       <c r="B173" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C173" s="5" t="s">
-        <v>12</v>
+      <c r="C173" s="5">
+        <v>1</v>
       </c>
       <c r="D173" s="5"/>
       <c r="E173" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:18:38
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -2062,8 +2062,8 @@
       <c r="B162" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C162" s="5" t="s">
-        <v>12</v>
+      <c r="C162" s="5">
+        <v>1</v>
       </c>
       <c r="D162" s="5"/>
       <c r="E162" s="5"/>
@@ -2073,8 +2073,8 @@
       <c r="B163" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C163" s="5" t="s">
-        <v>12</v>
+      <c r="C163" s="5">
+        <v>1</v>
       </c>
       <c r="D163" s="5"/>
       <c r="E163" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:19:02
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -1977,8 +1977,8 @@
       <c r="B153" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C153" s="5" t="s">
-        <v>12</v>
+      <c r="C153" s="5">
+        <v>1</v>
       </c>
       <c r="D153" s="5"/>
       <c r="E153" s="5"/>
@@ -1988,8 +1988,8 @@
       <c r="B154" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C154" s="5" t="s">
-        <v>12</v>
+      <c r="C154" s="5">
+        <v>1</v>
       </c>
       <c r="D154" s="5"/>
       <c r="E154" s="5"/>
@@ -1999,8 +1999,8 @@
       <c r="B155" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C155" s="5" t="s">
-        <v>12</v>
+      <c r="C155" s="5">
+        <v>1</v>
       </c>
       <c r="D155" s="5"/>
       <c r="E155" s="5"/>
@@ -2084,14 +2084,14 @@
       <c r="B164" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C164" s="5" t="s">
-        <v>12</v>
+      <c r="C164" s="5">
+        <v>1</v>
       </c>
       <c r="D164" s="5">
         <v>1</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:20:01
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -1892,8 +1892,8 @@
       <c r="B144" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C144" s="5" t="s">
-        <v>12</v>
+      <c r="C144" s="5">
+        <v>1</v>
       </c>
       <c r="D144" s="5"/>
       <c r="E144" s="5"/>
@@ -1903,8 +1903,8 @@
       <c r="B145" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C145" s="5" t="s">
-        <v>12</v>
+      <c r="C145" s="5">
+        <v>1</v>
       </c>
       <c r="D145" s="5"/>
       <c r="E145" s="5"/>
@@ -1914,8 +1914,8 @@
       <c r="B146" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C146" s="5" t="s">
-        <v>12</v>
+      <c r="C146" s="5">
+        <v>1</v>
       </c>
       <c r="D146" s="5"/>
       <c r="E146" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:22:21
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -1807,8 +1807,8 @@
       <c r="B135" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C135" s="5" t="s">
-        <v>12</v>
+      <c r="C135" s="5">
+        <v>1</v>
       </c>
       <c r="D135" s="5"/>
       <c r="E135" s="5"/>
@@ -1818,8 +1818,8 @@
       <c r="B136" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C136" s="5" t="s">
-        <v>12</v>
+      <c r="C136" s="5">
+        <v>1</v>
       </c>
       <c r="D136" s="5"/>
       <c r="E136" s="5"/>
@@ -1829,8 +1829,8 @@
       <c r="B137" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C137" s="5" t="s">
-        <v>12</v>
+      <c r="C137" s="5">
+        <v>1</v>
       </c>
       <c r="D137" s="5"/>
       <c r="E137" s="5"/>
@@ -2931,12 +2931,8 @@
       <c r="C252" s="5">
         <v>1</v>
       </c>
-      <c r="D252" s="5">
-        <v>1</v>
-      </c>
-      <c r="E252" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="D252" s="5"/>
+      <c r="E252" s="5"/>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:33:06
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -2891,9 +2891,7 @@
       <c r="B249" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C249" s="5">
-        <v>2</v>
-      </c>
+      <c r="C249" s="5"/>
       <c r="D249" s="5"/>
       <c r="E249" s="5"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour du suivi — 25/10/2026 15:33:09
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -2891,7 +2891,9 @@
       <c r="B249" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C249" s="5"/>
+      <c r="C249" s="5">
+        <v>1</v>
+      </c>
       <c r="D249" s="5"/>
       <c r="E249" s="5"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 10:41:39
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -461,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E254"/>
+  <dimension ref="A1:E263"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2956,8 +2956,91 @@
       <c r="D254" s="5"/>
       <c r="E254" s="5"/>
     </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A257" s="3">
+        <v>46321</v>
+      </c>
+      <c r="B257" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C257" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D257" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E257" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A258" s="3"/>
+      <c r="B258" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C258" s="5">
+        <v>1</v>
+      </c>
+      <c r="D258" s="5"/>
+      <c r="E258" s="5"/>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A259" s="3"/>
+      <c r="B259" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C259" s="5">
+        <v>1</v>
+      </c>
+      <c r="D259" s="5"/>
+      <c r="E259" s="5"/>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A260" s="3"/>
+      <c r="B260" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C260" s="5">
+        <v>1</v>
+      </c>
+      <c r="D260" s="5"/>
+      <c r="E260" s="5"/>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A261" s="3"/>
+      <c r="B261" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C261" s="5">
+        <v>1</v>
+      </c>
+      <c r="D261" s="5"/>
+      <c r="E261" s="5"/>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A262" s="3"/>
+      <c r="B262" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C262" s="5">
+        <v>1</v>
+      </c>
+      <c r="D262" s="5"/>
+      <c r="E262" s="5"/>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A263" s="3"/>
+      <c r="B263" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C263" s="5">
+        <v>1</v>
+      </c>
+      <c r="D263" s="5"/>
+      <c r="E263" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="29">
     <mergeCell ref="A4:A11"/>
     <mergeCell ref="A14:A20"/>
     <mergeCell ref="A23:A29"/>
@@ -2986,6 +3069,7 @@
     <mergeCell ref="A230:A236"/>
     <mergeCell ref="A239:A245"/>
     <mergeCell ref="A248:A254"/>
+    <mergeCell ref="A257:A263"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 10:43:11
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="18">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -461,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E263"/>
+  <dimension ref="A1:E264"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -2956,6 +2956,8 @@
       <c r="D254" s="5"/>
       <c r="E254" s="5"/>
     </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="3">
         <v>46321</v>
@@ -3038,6 +3040,15 @@
       </c>
       <c r="D263" s="5"/>
       <c r="E263" s="5"/>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A264" s="3"/>
+      <c r="B264" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C264" s="5"/>
+      <c r="D264" s="5"/>
+      <c r="E264" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="29">
@@ -3069,7 +3080,7 @@
     <mergeCell ref="A230:A236"/>
     <mergeCell ref="A239:A245"/>
     <mergeCell ref="A248:A254"/>
-    <mergeCell ref="A257:A263"/>
+    <mergeCell ref="A257:A264"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 10:43:16
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>0min</t>
+  </si>
+  <si>
+    <t>Travail</t>
   </si>
 </sst>
 </file>
@@ -3044,7 +3047,7 @@
     <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="3"/>
       <c r="B264" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C264" s="5"/>
       <c r="D264" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 10:43:18
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -3049,7 +3049,9 @@
       <c r="B264" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C264" s="5"/>
+      <c r="C264" s="5">
+        <v>1</v>
+      </c>
       <c r="D264" s="5"/>
       <c r="E264" s="5"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 10:43:30
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="19">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E264"/>
+  <dimension ref="A1:E265"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" defaultColWidth="9.06640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.19921875" style="1" customWidth="1"/>
@@ -3054,6 +3054,15 @@
       </c>
       <c r="D264" s="5"/>
       <c r="E264" s="5"/>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A265" s="3"/>
+      <c r="B265" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C265" s="5"/>
+      <c r="D265" s="5"/>
+      <c r="E265" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="29">
@@ -3085,7 +3094,7 @@
     <mergeCell ref="A230:A236"/>
     <mergeCell ref="A239:A245"/>
     <mergeCell ref="A248:A254"/>
-    <mergeCell ref="A257:A264"/>
+    <mergeCell ref="A257:A265"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 10:43:33
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>Travail</t>
+  </si>
+  <si>
+    <t>NouvelleSalat action</t>
   </si>
 </sst>
 </file>
@@ -3058,7 +3061,7 @@
     <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="3"/>
       <c r="B265" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C265" s="5"/>
       <c r="D265" s="5"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 10:43:43
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -3063,7 +3063,9 @@
       <c r="B265" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C265" s="5"/>
+      <c r="C265" s="5">
+        <v>5</v>
+      </c>
       <c r="D265" s="5"/>
       <c r="E265" s="5"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 16:38:04
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -3055,8 +3055,12 @@
       <c r="C264" s="5">
         <v>1</v>
       </c>
-      <c r="D264" s="5"/>
-      <c r="E264" s="5"/>
+      <c r="D264" s="5">
+        <v>1</v>
+      </c>
+      <c r="E264" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 18:40:59
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -3022,8 +3022,12 @@
       <c r="C261" s="5">
         <v>1</v>
       </c>
-      <c r="D261" s="5"/>
-      <c r="E261" s="5"/>
+      <c r="D261" s="5">
+        <v>1</v>
+      </c>
+      <c r="E261" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 18:57:30
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -3074,8 +3074,12 @@
       <c r="C265" s="5">
         <v>5</v>
       </c>
-      <c r="D265" s="5"/>
-      <c r="E265" s="5"/>
+      <c r="D265" s="5">
+        <v>3</v>
+      </c>
+      <c r="E265" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="29">

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 19:25:43
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -3011,8 +3011,12 @@
       <c r="C260" s="5">
         <v>1</v>
       </c>
-      <c r="D260" s="5"/>
-      <c r="E260" s="5"/>
+      <c r="D260" s="5">
+        <v>1</v>
+      </c>
+      <c r="E260" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="3"/>

</xml_diff>

<commit_message>
Mise à jour du suivi — 26/10/2026 21:09:26
</commit_message>
<xml_diff>
--- a/Plan_V1.xlsx
+++ b/Plan_V1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="20">
   <si>
     <r>
       <t xml:space="preserve">📅 </t>
@@ -3052,8 +3052,12 @@
       <c r="C263" s="5">
         <v>1</v>
       </c>
-      <c r="D263" s="5"/>
-      <c r="E263" s="5"/>
+      <c r="D263" s="5">
+        <v>1</v>
+      </c>
+      <c r="E263" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="3"/>

</xml_diff>